<commit_message>
Notes in response to review by Peter. Defered removal of Planned from PlannedProcessStep and mfgProcessMachine -> mfgProcessSystem until all isolated changes are complete.
</commit_message>
<xml_diff>
--- a/ShortHands.xlsx
+++ b/ShortHands.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/akitt/Code/AM-CDM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexkitt/Code/AM-CDM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6F5579F-6542-DD49-AFDE-B6AAE088FC79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{452EB892-2FD6-BF43-B01A-9EFEF5DAB07D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="32000" windowHeight="18000" xr2:uid="{D075A580-C83A-6248-82D1-7622755D1633}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="32000" windowHeight="18000" xr2:uid="{D075A580-C83A-6248-82D1-7622755D1633}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="147">
   <si>
     <t>Class</t>
   </si>
@@ -514,6 +514,12 @@
   </si>
   <si>
     <t>mfgSpec</t>
+  </si>
+  <si>
+    <t>MaterialTransfer</t>
+  </si>
+  <si>
+    <t>transfer</t>
   </si>
 </sst>
 </file>
@@ -919,7 +925,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD1FF16C-185E-F44C-A775-DF5CC764CA70}">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.1640625" bestFit="1" customWidth="1"/>
@@ -1217,13 +1223,13 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>145</v>
       </c>
       <c r="C28" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -1231,10 +1237,10 @@
         <v>47</v>
       </c>
       <c r="B29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C29" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -1242,10 +1248,10 @@
         <v>47</v>
       </c>
       <c r="B30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C30" t="s">
-        <v>78</v>
+        <v>144</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -1253,7 +1259,10 @@
         <v>47</v>
       </c>
       <c r="B31" t="s">
-        <v>51</v>
+        <v>50</v>
+      </c>
+      <c r="C31" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -1261,10 +1270,7 @@
         <v>47</v>
       </c>
       <c r="B32" t="s">
-        <v>52</v>
-      </c>
-      <c r="C32" t="s">
-        <v>76</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -1272,7 +1278,10 @@
         <v>47</v>
       </c>
       <c r="B33" t="s">
-        <v>53</v>
+        <v>52</v>
+      </c>
+      <c r="C33" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -1280,7 +1289,7 @@
         <v>47</v>
       </c>
       <c r="B34" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -1288,10 +1297,7 @@
         <v>47</v>
       </c>
       <c r="B35" t="s">
-        <v>55</v>
-      </c>
-      <c r="C35" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -1299,15 +1305,18 @@
         <v>47</v>
       </c>
       <c r="B36" t="s">
-        <v>56</v>
+        <v>55</v>
+      </c>
+      <c r="C36" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -1315,10 +1324,7 @@
         <v>57</v>
       </c>
       <c r="B38" t="s">
-        <v>59</v>
-      </c>
-      <c r="C38" t="s">
-        <v>82</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -1326,10 +1332,10 @@
         <v>57</v>
       </c>
       <c r="B39" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -1337,10 +1343,10 @@
         <v>57</v>
       </c>
       <c r="B40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -1348,10 +1354,10 @@
         <v>57</v>
       </c>
       <c r="B41" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -1359,10 +1365,10 @@
         <v>57</v>
       </c>
       <c r="B42" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C42" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -1370,10 +1376,10 @@
         <v>57</v>
       </c>
       <c r="B43" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C43" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -1381,7 +1387,10 @@
         <v>57</v>
       </c>
       <c r="B44" t="s">
-        <v>65</v>
+        <v>64</v>
+      </c>
+      <c r="C44" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -1389,10 +1398,7 @@
         <v>57</v>
       </c>
       <c r="B45" t="s">
-        <v>66</v>
-      </c>
-      <c r="C45" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -1400,10 +1406,10 @@
         <v>57</v>
       </c>
       <c r="B46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -1411,21 +1417,21 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C47" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="B48" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="C48" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -1433,7 +1439,10 @@
         <v>93</v>
       </c>
       <c r="B49" t="s">
-        <v>95</v>
+        <v>94</v>
+      </c>
+      <c r="C49" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -1441,7 +1450,7 @@
         <v>93</v>
       </c>
       <c r="B50" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -1449,10 +1458,7 @@
         <v>93</v>
       </c>
       <c r="B51" t="s">
-        <v>97</v>
-      </c>
-      <c r="C51" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -1460,7 +1466,10 @@
         <v>93</v>
       </c>
       <c r="B52" t="s">
-        <v>98</v>
+        <v>97</v>
+      </c>
+      <c r="C52" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -1468,10 +1477,7 @@
         <v>93</v>
       </c>
       <c r="B53" t="s">
-        <v>99</v>
-      </c>
-      <c r="C53" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -1479,10 +1485,10 @@
         <v>93</v>
       </c>
       <c r="B54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C54" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -1490,21 +1496,21 @@
         <v>93</v>
       </c>
       <c r="B55" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C55" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="B56" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="C56" t="s">
-        <v>69</v>
+        <v>106</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -1512,10 +1518,10 @@
         <v>69</v>
       </c>
       <c r="B57" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C57" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -1523,10 +1529,10 @@
         <v>69</v>
       </c>
       <c r="B58" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C58" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -1534,7 +1540,10 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="C59" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
@@ -1542,7 +1551,7 @@
         <v>69</v>
       </c>
       <c r="B60" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
@@ -1550,18 +1559,15 @@
         <v>69</v>
       </c>
       <c r="B61" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>107</v>
+        <v>69</v>
       </c>
       <c r="B62" t="s">
-        <v>108</v>
-      </c>
-      <c r="C62" t="s">
-        <v>107</v>
+        <v>75</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
@@ -1569,10 +1575,10 @@
         <v>107</v>
       </c>
       <c r="B63" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C63" t="s">
-        <v>128</v>
+        <v>107</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
@@ -1580,10 +1586,10 @@
         <v>107</v>
       </c>
       <c r="B64" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C64" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
@@ -1591,10 +1597,10 @@
         <v>107</v>
       </c>
       <c r="B65" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C65" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
@@ -1602,10 +1608,10 @@
         <v>107</v>
       </c>
       <c r="B66" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C66" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
@@ -1613,10 +1619,10 @@
         <v>107</v>
       </c>
       <c r="B67" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C67" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
@@ -1624,10 +1630,10 @@
         <v>107</v>
       </c>
       <c r="B68" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C68" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -1635,10 +1641,10 @@
         <v>107</v>
       </c>
       <c r="B69" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C69" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
@@ -1646,10 +1652,10 @@
         <v>107</v>
       </c>
       <c r="B70" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C70" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -1657,10 +1663,10 @@
         <v>107</v>
       </c>
       <c r="B71" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C71" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
@@ -1668,10 +1674,10 @@
         <v>107</v>
       </c>
       <c r="B72" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C72" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
@@ -1679,7 +1685,10 @@
         <v>107</v>
       </c>
       <c r="B73" t="s">
-        <v>119</v>
+        <v>118</v>
+      </c>
+      <c r="C73" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -1687,7 +1696,7 @@
         <v>107</v>
       </c>
       <c r="B74" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -1695,7 +1704,7 @@
         <v>107</v>
       </c>
       <c r="B75" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -1703,7 +1712,7 @@
         <v>107</v>
       </c>
       <c r="B76" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
@@ -1711,10 +1720,7 @@
         <v>107</v>
       </c>
       <c r="B77" t="s">
-        <v>123</v>
-      </c>
-      <c r="C77" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
@@ -1722,10 +1728,10 @@
         <v>107</v>
       </c>
       <c r="B78" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C78" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
@@ -1733,10 +1739,10 @@
         <v>107</v>
       </c>
       <c r="B79" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C79" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
@@ -1744,10 +1750,10 @@
         <v>107</v>
       </c>
       <c r="B80" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C80" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -1755,9 +1761,20 @@
         <v>107</v>
       </c>
       <c r="B81" t="s">
+        <v>126</v>
+      </c>
+      <c r="C81" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>107</v>
+      </c>
+      <c r="B82" t="s">
         <v>127</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C82" t="s">
         <v>138</v>
       </c>
     </row>

</xml_diff>